<commit_message>
Implemented node_hunter, member_scraper, and presser_scraper functions. Still require bug squashing and testing but working for barrymoore.house.gov
</commit_message>
<xml_diff>
--- a/nodes.xlsx
+++ b/nodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zayne\GitRepos\PresserScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21BDE8E-8A92-4104-B7A8-4DCDC565877C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863D6D0F-10CF-498B-B924-717FB9D76C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19305" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
+    <workbookView xWindow="11160" yWindow="5325" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="64">
   <si>
     <t>template</t>
   </si>
@@ -60,9 +60,6 @@
     <t>.col-auto:nth-child(1)</t>
   </si>
   <si>
-    <t>/page/</t>
-  </si>
-  <si>
     <t>.published</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
     <t>h2</t>
   </si>
   <si>
-    <t>texts</t>
-  </si>
-  <si>
     <t>.page-content</t>
   </si>
   <si>
@@ -223,13 +217,25 @@
   </si>
   <si>
     <t>This spreadsheet aims to provide a comprehensive list of nodes (CSS or less commonly xpath) to reach the links, dates, and titles of press releases from members' house.gov sites.</t>
+  </si>
+  <si>
+    <t>page/</t>
+  </si>
+  <si>
+    <t>.evo-content</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>.evo-press-release__field-evo-issues</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +245,14 @@
     </font>
     <font>
       <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -265,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -273,6 +287,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -607,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDF2318D-EAE3-4B24-AE0D-096822628925}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
@@ -616,34 +631,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
-        <v>13</v>
+      <c r="E1" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -654,7 +669,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
@@ -662,19 +677,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -682,38 +694,38 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
@@ -721,689 +733,721 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
+        <v>5</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="C10" t="s">
         <v>54</v>
       </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D12" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
         <v>9</v>
       </c>
-      <c r="B16" t="s">
-        <v>25</v>
-      </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D25" t="s">
-        <v>27</v>
+        <v>1</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D26" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D27" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D29" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D30" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D31" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" t="s">
         <v>17</v>
       </c>
-      <c r="B32" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D32" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="C37" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" t="s">
+        <v>52</v>
+      </c>
+      <c r="D39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42" t="s">
+        <v>52</v>
+      </c>
+      <c r="D42" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C43" t="s">
+        <v>52</v>
+      </c>
+      <c r="D43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>8</v>
+      </c>
+      <c r="B45" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" t="s">
+        <v>52</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B46" t="s">
         <v>9</v>
       </c>
-      <c r="B33" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" t="s">
-        <v>54</v>
-      </c>
-      <c r="D33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>40</v>
-      </c>
-      <c r="B34" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D34" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" t="s">
-        <v>54</v>
-      </c>
-      <c r="D35" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
-        <v>4</v>
-      </c>
-      <c r="C36" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>5</v>
-      </c>
-      <c r="B37" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" t="s">
-        <v>54</v>
-      </c>
-      <c r="D37" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>11</v>
-      </c>
-      <c r="B38" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" t="s">
-        <v>54</v>
-      </c>
-      <c r="D38" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="C46" t="s">
+        <v>52</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>8</v>
+      </c>
+      <c r="B47" t="s">
         <v>9</v>
       </c>
-      <c r="B39" t="s">
-        <v>44</v>
-      </c>
-      <c r="C39" t="s">
-        <v>54</v>
-      </c>
-      <c r="D39" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>3</v>
-      </c>
-      <c r="B41" t="s">
-        <v>4</v>
-      </c>
-      <c r="C41" t="s">
-        <v>53</v>
-      </c>
-      <c r="D41" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>5</v>
-      </c>
-      <c r="B42" t="s">
-        <v>45</v>
-      </c>
-      <c r="C42" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" t="s">
-        <v>54</v>
-      </c>
-      <c r="D43" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>40</v>
-      </c>
-      <c r="B44" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>40</v>
-      </c>
-      <c r="B45" t="s">
+      <c r="C47" t="s">
+        <v>52</v>
+      </c>
+      <c r="D47" t="s">
         <v>48</v>
       </c>
-      <c r="C45" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>3</v>
-      </c>
-      <c r="B46" t="s">
-        <v>4</v>
-      </c>
-      <c r="C46" t="s">
-        <v>53</v>
-      </c>
-      <c r="D46" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>5</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C47" t="s">
-        <v>56</v>
-      </c>
-      <c r="D47" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="C49" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D49" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C50" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D51" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>50</v>
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B53" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="C53" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B54" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="C54" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D54" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B55" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="C55" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D55" t="s">
-        <v>50</v>
-      </c>
-      <c r="E55" t="s">
-        <v>20</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>8</v>
+      </c>
+      <c r="B56" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56" t="s">
+        <v>52</v>
+      </c>
+      <c r="D56" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E56">
+    <sortCondition ref="A2:A56"/>
+    <sortCondition ref="B2:B56"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1418,7 +1462,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="319.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added edge case scraper
</commit_message>
<xml_diff>
--- a/nodes.xlsx
+++ b/nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zayne\GitRepos\PresserScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863D6D0F-10CF-498B-B924-717FB9D76C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B184D871-A15D-419E-B42A-CBA2DF143AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11160" yWindow="5325" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="62">
   <si>
     <t>template</t>
   </si>
@@ -196,12 +196,6 @@
   </si>
   <si>
     <t>css</t>
-  </si>
-  <si>
-    <t>//*[contains(concat( \" \", @class, \" \" ), concat( \" \", \"col-auto\", \" \" ))]</t>
-  </si>
-  <si>
-    <t>xpath</t>
   </si>
   <si>
     <t>?PageNum_rs=</t>
@@ -279,11 +273,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -631,19 +622,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -652,7 +643,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
         <v>52</v>
@@ -759,32 +750,32 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>53</v>
+      <c r="B10" t="s">
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -792,13 +783,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>52</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -806,13 +797,13 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s">
         <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -820,7 +811,7 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C14" t="s">
         <v>52</v>
@@ -840,7 +831,7 @@
         <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -848,13 +839,13 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
         <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -862,13 +853,13 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
         <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -876,13 +867,13 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
         <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -890,13 +881,13 @@
         <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
         <v>52</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -910,7 +901,7 @@
         <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -924,7 +915,7 @@
         <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -932,27 +923,27 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C22" t="s">
         <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -960,13 +951,13 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
       </c>
       <c r="D24" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -974,16 +965,13 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="C25" t="s">
         <v>51</v>
       </c>
       <c r="D25" t="s">
-        <v>1</v>
-      </c>
-      <c r="E25" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -991,16 +979,13 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
         <v>51</v>
       </c>
       <c r="D26" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1014,7 +999,7 @@
         <v>51</v>
       </c>
       <c r="D27" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1022,13 +1007,13 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="C28" t="s">
         <v>51</v>
       </c>
       <c r="D28" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1036,13 +1021,16 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="C29" t="s">
         <v>51</v>
       </c>
       <c r="D29" t="s">
-        <v>47</v>
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1050,27 +1038,27 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="C30" t="s">
         <v>51</v>
       </c>
       <c r="D30" t="s">
-        <v>48</v>
+        <v>26</v>
+      </c>
+      <c r="E30" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1078,7 +1066,7 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
         <v>52</v>
@@ -1123,13 +1111,13 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C35" t="s">
         <v>52</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1137,16 +1125,13 @@
         <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
         <v>52</v>
       </c>
       <c r="D36" t="s">
-        <v>1</v>
-      </c>
-      <c r="E36" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1154,13 +1139,16 @@
         <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C37" t="s">
         <v>52</v>
       </c>
       <c r="D37" t="s">
         <v>1</v>
+      </c>
+      <c r="E37" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1168,13 +1156,13 @@
         <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
         <v>52</v>
       </c>
       <c r="D38" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1182,13 +1170,13 @@
         <v>16</v>
       </c>
       <c r="B39" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="C39" t="s">
         <v>52</v>
       </c>
       <c r="D39" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1196,13 +1184,13 @@
         <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="C40" t="s">
         <v>52</v>
       </c>
       <c r="D40" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1224,7 +1212,7 @@
         <v>16</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C42" t="s">
         <v>52</v>
@@ -1238,7 +1226,7 @@
         <v>16</v>
       </c>
       <c r="B43" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C43" t="s">
         <v>52</v>
@@ -1266,13 +1254,10 @@
         <v>8</v>
       </c>
       <c r="B45" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="C45" t="s">
         <v>52</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1280,7 +1265,7 @@
         <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
@@ -1300,7 +1285,7 @@
         <v>52</v>
       </c>
       <c r="D47" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1308,13 +1293,13 @@
         <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="C48" t="s">
         <v>52</v>
       </c>
       <c r="D48" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1322,13 +1307,13 @@
         <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C49" t="s">
         <v>52</v>
       </c>
       <c r="D49" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1336,13 +1321,13 @@
         <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C50" t="s">
         <v>52</v>
       </c>
       <c r="D50" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -1350,13 +1335,13 @@
         <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="C51" t="s">
         <v>52</v>
       </c>
       <c r="D51" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1364,16 +1349,13 @@
         <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="C52" t="s">
         <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>1</v>
-      </c>
-      <c r="E52" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -1381,13 +1363,16 @@
         <v>8</v>
       </c>
       <c r="B53" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="C53" t="s">
         <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>41</v>
+        <v>1</v>
+      </c>
+      <c r="E53" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -1395,13 +1380,13 @@
         <v>8</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C54" t="s">
         <v>52</v>
       </c>
       <c r="D54" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1409,7 +1394,7 @@
         <v>8</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C55" t="s">
         <v>52</v>
@@ -1423,7 +1408,7 @@
         <v>8</v>
       </c>
       <c r="B56" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C56" t="s">
         <v>52</v>
@@ -1434,19 +1419,22 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="B57" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="C57" t="s">
         <v>52</v>
       </c>
+      <c r="D57" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E56">
-    <sortCondition ref="A2:A56"/>
-    <sortCondition ref="B2:B56"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E57">
+    <sortCondition ref="A2:A57"/>
+    <sortCondition ref="B2:B57"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1461,8 +1449,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="319.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>59</v>
+      <c r="A1" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improvements to date detection and formatting
</commit_message>
<xml_diff>
--- a/nodes.xlsx
+++ b/nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zayne\GitRepos\PresserScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B184D871-A15D-419E-B42A-CBA2DF143AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038B3D8C-E4A3-4844-BD17-E971B5F588CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="63">
   <si>
     <t>template</t>
   </si>
@@ -57,9 +57,6 @@
     <t>dates</t>
   </si>
   <si>
-    <t>.col-auto:nth-child(1)</t>
-  </si>
-  <si>
     <t>.published</t>
   </si>
   <si>
@@ -223,6 +220,12 @@
   </si>
   <si>
     <t>.evo-press-release__field-evo-issues</t>
+  </si>
+  <si>
+    <t>.col-auto</t>
+  </si>
+  <si>
+    <t>.views-row .font-weight-bold a</t>
   </si>
 </sst>
 </file>
@@ -626,16 +629,16 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -643,13 +646,13 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -657,10 +660,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
@@ -671,13 +674,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -685,13 +688,13 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -699,13 +702,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -713,13 +716,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -727,13 +730,13 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -741,66 +744,66 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
@@ -808,128 +811,128 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -937,13 +940,13 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -954,10 +957,10 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D24" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -968,10 +971,10 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -982,7 +985,7 @@
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D26" t="s">
         <v>47</v>
@@ -993,13 +996,13 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1007,13 +1010,16 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="E28" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1021,254 +1027,251 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C30" t="s">
         <v>51</v>
-      </c>
-      <c r="D30" t="s">
-        <v>26</v>
-      </c>
-      <c r="E30" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+      <c r="D31" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D32" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D35" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D36" t="s">
-        <v>26</v>
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D37" t="s">
-        <v>1</v>
-      </c>
-      <c r="E37" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" t="s">
         <v>16</v>
       </c>
-      <c r="B38" t="s">
-        <v>59</v>
-      </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D38" t="s">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" t="s">
         <v>16</v>
       </c>
-      <c r="B39" t="s">
-        <v>17</v>
-      </c>
       <c r="C39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D39" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" t="s">
         <v>16</v>
       </c>
-      <c r="B40" t="s">
-        <v>17</v>
-      </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D40" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B41" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C41" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D41" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D42" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D43" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B44" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
-      </c>
-      <c r="D44" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B45" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" t="s">
         <v>8</v>
       </c>
-      <c r="B46" t="s">
-        <v>15</v>
-      </c>
       <c r="C46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D46" t="s">
         <v>1</v>
@@ -1276,165 +1279,162 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
         <v>8</v>
       </c>
-      <c r="B47" t="s">
-        <v>9</v>
-      </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D47" t="s">
-        <v>1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B48" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D48" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B49" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D49" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B50" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D50" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B51" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D51" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B52" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D52" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B53" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D53" t="s">
-        <v>1</v>
-      </c>
-      <c r="E53" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B54" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D54" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B55" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D55" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B56" t="s">
         <v>34</v>
       </c>
       <c r="C56" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D56" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B57" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>52</v>
-      </c>
-      <c r="D57" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E57">
-    <sortCondition ref="A2:A57"/>
-    <sortCondition ref="B2:B57"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E56">
+    <sortCondition ref="A2:A56"/>
+    <sortCondition ref="B2:B56"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1450,7 +1450,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="319.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test of full domain list and bug squashing
</commit_message>
<xml_diff>
--- a/nodes.xlsx
+++ b/nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zayne\GitRepos\PresserScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038B3D8C-E4A3-4844-BD17-E971B5F588CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D673F936-8926-4890-90A5-E9FBBACFBE11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="22110" windowHeight="15555" xr2:uid="{218D3161-3301-4141-9F88-B4178F9F1B21}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="63">
   <si>
     <t>template</t>
   </si>
@@ -616,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDF2318D-EAE3-4B24-AE0D-096822628925}">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
@@ -1428,6 +1428,17 @@
         <v>62</v>
       </c>
       <c r="C57" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" t="s">
+        <v>62</v>
+      </c>
+      <c r="C58" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>